<commit_message>
Set Spanish material schedule to Beijing midnight and recognize Spanish row alias
</commit_message>
<xml_diff>
--- a/assets_es_20261026/titles.xlsx
+++ b/assets_es_20261026/titles.xlsx
@@ -522,7 +522,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>17:00（北京时间）</t>
+          <t>00:00（北京时间）</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -589,7 +589,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>17:00（北京时间）</t>
+          <t>00:00（北京时间）</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -656,7 +656,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>17:00（北京时间）</t>
+          <t>00:00（北京时间）</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -723,7 +723,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>17:00（北京时间）</t>
+          <t>00:00（北京时间）</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -790,7 +790,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>17:00（北京时间）</t>
+          <t>00:00（北京时间）</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -857,7 +857,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>17:00（北京时间）</t>
+          <t>00:00（北京时间）</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -924,7 +924,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>17:00（北京时间）</t>
+          <t>00:00（北京时间）</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>17:00（北京时间）</t>
+          <t>00:00（北京时间）</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1058,7 +1058,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>17:00（北京时间）</t>
+          <t>00:00（北京时间）</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1125,7 +1125,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>17:00（北京时间）</t>
+          <t>00:00（北京时间）</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1192,7 +1192,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>17:00（北京时间）</t>
+          <t>00:00（北京时间）</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1259,7 +1259,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>17:00（北京时间）</t>
+          <t>00:00（北京时间）</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1326,7 +1326,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>17:00（北京时间）</t>
+          <t>00:00（北京时间）</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1393,7 +1393,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>17:00（北京时间）</t>
+          <t>00:00（北京时间）</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1460,7 +1460,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>17:00（北京时间）</t>
+          <t>00:00（北京时间）</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1527,7 +1527,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>17:00（北京时间）</t>
+          <t>00:00（北京时间）</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1594,7 +1594,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>17:00（北京时间）</t>
+          <t>00:00（北京时间）</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1661,7 +1661,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>17:00（北京时间）</t>
+          <t>00:00（北京时间）</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -1728,7 +1728,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>17:00（北京时间）</t>
+          <t>00:00（北京时间）</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1795,7 +1795,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>17:00（北京时间）</t>
+          <t>00:00（北京时间）</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -1862,7 +1862,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>17:00（北京时间）</t>
+          <t>00:00（北京时间）</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -1956,7 +1956,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1983,7 +1983,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26—2026-11-15，每天北京时间17:00</t>
+          <t>2026-10-26—2026-11-15，每天北京时间00:00</t>
         </is>
       </c>
     </row>
@@ -2068,6 +2068,30 @@
       <c r="B9" s="2" t="inlineStr">
         <is>
           <t>保留YouTube原说明，仅末行追加对应剧集代码</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>本次时间更新</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>西班牙=西语；所有日期不变，每天北京时间00:00；只更新本机素材，不自动修改线上已定时视频。</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>禁播提醒</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>11月5日《从蚁王开始吞噬成神》在最新资源表标为禁播，请跳过；本次未更换该剧。</t>
         </is>
       </c>
     </row>

</xml_diff>